<commit_message>
Snapshot current working state: LinkedIn reportable dataset pipeline, report-category features, Apify sync, admin/public portal updates, and dataset snapshots
</commit_message>
<xml_diff>
--- a/data/exports/tce_activity_intelligence.xlsx
+++ b/data/exports/tce_activity_intelligence.xlsx
@@ -23,16 +23,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,21 +48,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,17 +423,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>year_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>total_activities</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
@@ -527,26 +515,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>department_code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>department_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>involvement_count</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>primary_count</t>
         </is>
@@ -699,12 +687,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>FASH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Fashion Technology</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -717,12 +705,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MATH</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Applied Mathematics and Computational Sciences</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -735,12 +723,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>MATH</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Management Studies</t>
+          <t>Applied Mathematics and Computational Sciences</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -753,12 +741,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MCT</t>
+          <t>MATHS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mechatronics Engineering</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -771,12 +759,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MECH</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Management Studies</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -789,18 +777,54 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>MCT</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mechatronics Engineering</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MECH</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>PHY</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -832,32 +856,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>classification_count</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>primary_count</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>avg_confidence</t>
         </is>
@@ -880,7 +904,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -904,7 +928,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -914,21 +938,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ALUMNI</t>
+          <t>RESEARCH</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alumni Event</t>
+          <t>Research and Consultancy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Alumni meets and alumni engagement</t>
+          <t>Research projects, patents, publications, consultancy</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -938,17 +962,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAMPUS</t>
+          <t>ALUMNI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Campus Life</t>
+          <t>Alumni Event</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Admissions, campus facilities, general campus events</t>
+          <t>Alumni meets and alumni engagement</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -962,17 +986,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CLUB</t>
+          <t>CAMPUS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Clubs and Chapters</t>
+          <t>Campus Life</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Student clubs, professional chapters, society meets</t>
+          <t>Admissions, campus facilities, general campus events</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -986,17 +1010,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CONFERENCE</t>
+          <t>CLUB</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Conference</t>
+          <t>Clubs and Chapters</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>National/international conferences</t>
+          <t>Student clubs, professional chapters, society meets</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -1010,17 +1034,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CULTURAL</t>
+          <t>CONFERENCE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cultural Event</t>
+          <t>Conference</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cultural programs and celebrations</t>
+          <t>National/international conferences</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1034,17 +1058,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FDP</t>
+          <t>CULTURAL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Faculty Development Programme</t>
+          <t>Cultural Event</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Faculty development and upskilling programs</t>
+          <t>Cultural programs and celebrations</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1058,17 +1082,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GUEST_LECTURE</t>
+          <t>FDP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Guest Lecture</t>
+          <t>Faculty Development Programme</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invited lectures by experts</t>
+          <t>Faculty development and upskilling programs</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1082,17 +1106,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HACKATHON</t>
+          <t>GUEST_LECTURE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hackathon</t>
+          <t>Guest Lecture</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Coding and innovation hackathons</t>
+          <t>Invited lectures by experts</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1106,17 +1130,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INDUSTRY</t>
+          <t>HACKATHON</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Industry Collaboration</t>
+          <t>Hackathon</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MoUs, industry visits, industry collaborations</t>
+          <t>Coding and innovation hackathons</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1130,17 +1154,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>INTERNSHIP</t>
+          <t>INDUSTRY</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Industry Collaboration</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Student/faculty internships</t>
+          <t>MoUs, industry visits, industry collaborations</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1154,17 +1178,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NCC</t>
+          <t>INTERNSHIP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NCC Activity</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>National Cadet Corps activities</t>
+          <t>Student/faculty internships</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1178,17 +1202,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NSS</t>
+          <t>NCC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NSS Activity</t>
+          <t>NCC Activity</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>National Service Scheme activities</t>
+          <t>National Cadet Corps activities</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1202,17 +1226,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ORIENTATION</t>
+          <t>NSS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Orientation and Convocation</t>
+          <t>NSS Activity</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Orientation, induction, convocation, graduation</t>
+          <t>National Service Scheme activities</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1226,17 +1250,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OUTREACH</t>
+          <t>ORIENTATION</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Outreach and Extension</t>
+          <t>Orientation and Convocation</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Community service, extension, rural outreach</t>
+          <t>Orientation, induction, convocation, graduation</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1250,17 +1274,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PLACEMENT</t>
+          <t>OUTREACH</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Placement Activity</t>
+          <t>Outreach and Extension</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Placement drives, career guidance, training for placement</t>
+          <t>Community service, extension, rural outreach</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1274,17 +1298,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RESEARCH</t>
+          <t>PLACEMENT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Research and Consultancy</t>
+          <t>Placement Activity</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Research projects, patents, publications, consultancy</t>
+          <t>Placement drives, career guidance, training for placement</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1454,27 +1478,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>involvement_count</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>primary_count</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>avg_confidence</t>
         </is>
@@ -1483,16 +1507,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ALUMNI</t>
+          <t>STUDENTS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alumni</t>
+          <t>Students</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -1502,12 +1526,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>COMMUNITY</t>
+          <t>ALUMNI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Community and Society</t>
+          <t>Alumni</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1521,12 +1545,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FACULTY</t>
+          <t>COMMUNITY</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Community and Society</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1540,12 +1564,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GOVERNMENT</t>
+          <t>FACULTY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Government and Agencies</t>
+          <t>Faculty</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1559,12 +1583,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>INDUSTRY</t>
+          <t>GOVERNMENT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Government and Agencies</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1578,12 +1602,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PARENTS</t>
+          <t>INDUSTRY</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Parents</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1597,12 +1621,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>STAFF</t>
+          <t>PARENTS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Non-Teaching Staff</t>
+          <t>Parents</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1616,12 +1640,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>STUDENTS</t>
+          <t>STAFF</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Non-Teaching Staff</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1647,12 +1671,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>count</t>
         </is>
@@ -1673,22 +1697,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>filled</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ratio</t>
         </is>
@@ -1701,10 +1725,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -1717,13 +1741,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0.7143</v>
       </c>
     </row>
     <row r="4">
@@ -1733,13 +1757,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>0.375</v>
+        <v>0.8571</v>
       </c>
     </row>
     <row r="5">
@@ -1752,7 +1776,7 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -1768,7 +1792,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1784,7 +1808,7 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -1797,13 +1821,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0.7143</v>
       </c>
     </row>
     <row r="9">
@@ -1813,13 +1837,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>0.4286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>